<commit_message>
Fix map (CARTO now requires API key -> switch to OSM tiles); sync 5 new venues + 3 host picks from owner's guide update [2026-09-30]
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Villa_Nobby_Local_Guide.xlsx
+++ b/Villa_Nobby_Local_Guide.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="2"/>
@@ -2403,7 +2403,11 @@
           <t>Lunch</t>
         </is>
       </c>
-      <c r="H46" s="15" t="n"/>
+      <c r="H46" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="47" hidden="1">
       <c r="A47" s="3" t="inlineStr">
@@ -2450,32 +2454,32 @@
     <row r="48" hidden="1">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Sushi Train</t>
+          <t>Okazu Sushi Bar</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>@sushitrainmiamione</t>
+          <t>@okazu_sushibar</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Japanese Sushi</t>
+          <t>Lunch / Japanese</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>450m</t>
+          <t>2km</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>6 min</t>
+          <t>4 min</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>Walk</t>
+          <t>Drive</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -2488,27 +2492,27 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Okazu Sushi Bar</t>
+          <t>Costa Taco Burleigh</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>@okazu_sushibar</t>
+          <t>@costa_taco</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Lunch / Japanese</t>
+          <t>Lunch / Mexican</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>2km</t>
+          <t>2.1km</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>4 min</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -2521,37 +2525,41 @@
           <t>Lunch</t>
         </is>
       </c>
-      <c r="H49" s="3" t="n"/>
+      <c r="H49" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Costa Taco Burleigh</t>
+          <t>Miami Sub</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>@costa_taco</t>
+          <t>@miamisubs_goldcoast</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Lunch / Mexican</t>
+          <t>Lunch / Sandwiches</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>2.1km</t>
+          <t>400m</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>6 min</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>Drive</t>
+          <t>Walk</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -2559,22 +2567,26 @@
           <t>Lunch</t>
         </is>
       </c>
-      <c r="H50" s="15" t="n"/>
+      <c r="H50" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="51" hidden="1">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Miami Sub</t>
+          <t>Street Fryer</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>@miamisubs_goldcoast</t>
+          <t>@streetfryer</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Lunch / Sandwiches</t>
+          <t>Lunch / Thai</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -2597,17 +2609,17 @@
           <t>Lunch</t>
         </is>
       </c>
-      <c r="H51" s="15" t="n"/>
+      <c r="H51" s="3" t="n"/>
     </row>
     <row r="52" hidden="1">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Street Fryer</t>
+          <t>Limlay Thai</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>@streetfryer</t>
+          <t>@limlayrestaurant</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -2617,153 +2629,153 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>400m</t>
+          <t>2.1km</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>6 min</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="22" t="inlineStr">
+        <is>
+          <t>More Thai At Nobby</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>@morethai.restaurants</t>
+        </is>
+      </c>
+      <c r="C53" s="21" t="inlineStr">
+        <is>
+          <t>Lunch / Thai</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>2km</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>4 min</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="G53" s="21" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>Maman Bar &amp; Kitchen</t>
+        </is>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>@maman_barkitchen</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Mediterranean</t>
+        </is>
+      </c>
+      <c r="D54" s="21" t="inlineStr">
+        <is>
+          <t>2.1km</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
+          <t>Light Years</t>
+        </is>
+      </c>
+      <c r="B55" s="21" t="inlineStr">
+        <is>
+          <t>@lightyearsasiandiner</t>
+        </is>
+      </c>
+      <c r="C55" s="21" t="inlineStr">
+        <is>
+          <t>Modern Asian Fusion</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>350m</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
           <t>Walk</t>
         </is>
       </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>Limlay Thai</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>@limlayrestaurant</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>Lunch / Thai</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>2.1km</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="F53" s="3" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="G53" s="3" t="inlineStr">
+      <c r="G55" s="21" t="inlineStr">
         <is>
           <t>Dinner</t>
         </is>
       </c>
-      <c r="H53" s="3" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="22" t="inlineStr">
-        <is>
-          <t>More Thai At Nobby</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>@morethai.restaurants</t>
-        </is>
-      </c>
-      <c r="C54" s="21" t="inlineStr">
-        <is>
-          <t>Lunch / Thai</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>2km</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>4 min</t>
-        </is>
-      </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="G54" s="21" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="6" t="inlineStr">
-        <is>
-          <t>Maman Bar &amp; Kitchen</t>
-        </is>
-      </c>
-      <c r="B55" s="11" t="inlineStr">
-        <is>
-          <t>@maman_barkitchen</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="inlineStr">
-        <is>
-          <t>Mediterranean</t>
-        </is>
-      </c>
-      <c r="D55" s="21" t="inlineStr">
-        <is>
-          <t>2.1km</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>Dinner</t>
-        </is>
-      </c>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="H55" s="3" t="n"/>
     </row>
     <row r="56" hidden="1">
       <c r="A56" s="22" t="inlineStr">
         <is>
-          <t>Light Years</t>
+          <t>Jimmy Wah's</t>
         </is>
       </c>
       <c r="B56" s="21" t="inlineStr">
         <is>
-          <t>@lightyearsasiandiner</t>
+          <t>@jimmywahs.burleigh</t>
         </is>
       </c>
       <c r="C56" s="21" t="inlineStr">
@@ -2773,7 +2785,7 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>350m</t>
+          <t>2.1km</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
@@ -2783,7 +2795,7 @@
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Walk</t>
+          <t>Drive</t>
         </is>
       </c>
       <c r="G56" s="21" t="inlineStr">
@@ -2791,17 +2803,17 @@
           <t>Dinner</t>
         </is>
       </c>
-      <c r="H56" s="3" t="n"/>
+      <c r="H56" s="14" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="22" t="inlineStr">
         <is>
-          <t>Jimmy Wah's</t>
+          <t>Baby Mama</t>
         </is>
       </c>
       <c r="B57" s="21" t="inlineStr">
         <is>
-          <t>@jimmywahs.burleigh</t>
+          <t>@babymama_bymamasan</t>
         </is>
       </c>
       <c r="C57" s="21" t="inlineStr">
@@ -2811,12 +2823,12 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>2.1km</t>
+          <t>2km</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>4 min</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -2829,61 +2841,57 @@
           <t>Dinner</t>
         </is>
       </c>
-      <c r="H57" s="14" t="n"/>
+      <c r="H57" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="22" t="inlineStr">
         <is>
-          <t>Baby Mama</t>
+          <t>North Burleigh Surf Club</t>
         </is>
       </c>
       <c r="B58" s="21" t="inlineStr">
         <is>
-          <t>@babymama_bymamasan</t>
+          <t>@north_burleighslsc_supporters</t>
         </is>
       </c>
       <c r="C58" s="21" t="inlineStr">
         <is>
-          <t>Modern Asian Fusion</t>
+          <t>Pub / Dinner</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>2km</t>
+          <t>650m</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>4 min</t>
+          <t>9 min</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Drive</t>
+          <t>Walk</t>
         </is>
       </c>
       <c r="G58" s="21" t="inlineStr">
         <is>
-          <t>Dinner</t>
-        </is>
-      </c>
-      <c r="H58" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Drinks</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="n"/>
     </row>
     <row r="59" hidden="1">
       <c r="A59" s="22" t="inlineStr">
         <is>
-          <t>North Burleigh Surf Club</t>
-        </is>
-      </c>
-      <c r="B59" s="21" t="inlineStr">
-        <is>
-          <t>@north_burleighslsc_supporters</t>
-        </is>
-      </c>
+          <t>Miami Tavern</t>
+        </is>
+      </c>
+      <c r="B59" s="21" t="n"/>
       <c r="C59" s="21" t="inlineStr">
         <is>
           <t>Pub / Dinner</t>
@@ -2891,12 +2899,12 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>650m</t>
+          <t>850m</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>9 min</t>
+          <t>12 min</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -2909,94 +2917,97 @@
           <t>Drinks</t>
         </is>
       </c>
-      <c r="H59" s="3" t="n"/>
+      <c r="H59" s="14" t="n"/>
     </row>
     <row r="60" hidden="1">
       <c r="A60" s="22" t="inlineStr">
         <is>
-          <t>Miami Tavern</t>
-        </is>
-      </c>
-      <c r="B60" s="21" t="n"/>
-      <c r="C60" s="21" t="inlineStr">
-        <is>
-          <t>Pub / Dinner</t>
+          <t>Paloma Wine Bar</t>
+        </is>
+      </c>
+      <c r="B60" s="14" t="inlineStr">
+        <is>
+          <t>@palomawinebar</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>Wine Bar</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>850m</t>
+          <t>2.1km</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>12 min</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>Walk</t>
-        </is>
-      </c>
-      <c r="G60" s="21" t="inlineStr">
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
         <is>
           <t>Drinks</t>
         </is>
       </c>
-      <c r="H60" s="14" t="n"/>
+      <c r="H60" s="15" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="22" t="inlineStr">
         <is>
-          <t>Paloma Wine Bar</t>
-        </is>
-      </c>
-      <c r="B61" s="14" t="inlineStr">
-        <is>
-          <t>@palomawinebar</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>Wine Bar</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
+          <t>ConkaBar</t>
+        </is>
+      </c>
+      <c r="B61" s="20" t="inlineStr">
+        <is>
+          <t>@conkabar</t>
+        </is>
+      </c>
+      <c r="C61" s="21" t="inlineStr">
+        <is>
+          <t>Dinner / Mexican</t>
+        </is>
+      </c>
+      <c r="D61" s="21" t="inlineStr">
         <is>
           <t>2.1km</t>
         </is>
       </c>
-      <c r="E61" s="3" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="F61" s="3" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="inlineStr">
-        <is>
-          <t>Drinks</t>
-        </is>
-      </c>
-      <c r="H61" s="15" t="n"/>
+      <c r="E61" s="21" t="inlineStr">
+        <is>
+          <t>7 min</t>
+        </is>
+      </c>
+      <c r="F61" s="21" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="G61" s="21" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="22" t="inlineStr">
         <is>
-          <t>ConkaBar</t>
+          <t>Shoto</t>
         </is>
       </c>
       <c r="B62" s="20" t="inlineStr">
         <is>
-          <t>@conkabar</t>
+          <t>@shotodining</t>
         </is>
       </c>
       <c r="C62" s="21" t="inlineStr">
         <is>
-          <t>Dinner / Mexican</t>
+          <t>Dinner / Japanese</t>
         </is>
       </c>
       <c r="D62" s="21" t="inlineStr">
@@ -3017,43 +3028,48 @@
       <c r="G62" s="21" t="inlineStr">
         <is>
           <t>Dinner</t>
+        </is>
+      </c>
+      <c r="H62" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="22" t="inlineStr">
         <is>
-          <t>Shoto</t>
-        </is>
-      </c>
-      <c r="B63" s="20" t="inlineStr">
-        <is>
-          <t>@shotodining</t>
+          <t>Ace's Coffee</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>@acescoffee.miami</t>
         </is>
       </c>
       <c r="C63" s="21" t="inlineStr">
         <is>
-          <t>Dinner / Japanese</t>
+          <t>Breakfast / Coffee</t>
         </is>
       </c>
       <c r="D63" s="21" t="inlineStr">
         <is>
-          <t>2.1km</t>
+          <t>350m</t>
         </is>
       </c>
       <c r="E63" s="21" t="inlineStr">
         <is>
-          <t>7 min</t>
+          <t>4 min</t>
         </is>
       </c>
       <c r="F63" s="21" t="inlineStr">
         <is>
-          <t>Drive</t>
+          <t>Walk</t>
         </is>
       </c>
       <c r="G63" s="21" t="inlineStr">
         <is>
-          <t>Dinner</t>
+          <t>Breakfast &amp; Cafés</t>
         </is>
       </c>
       <c r="H63" s="16" t="inlineStr">
@@ -3065,121 +3081,121 @@
     <row r="64" hidden="1">
       <c r="A64" s="22" t="inlineStr">
         <is>
-          <t>Ace's Coffee</t>
+          <t>Blend Greenness</t>
         </is>
       </c>
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t>@acescoffee.miami</t>
-        </is>
-      </c>
-      <c r="C64" s="21" t="inlineStr">
-        <is>
-          <t>Breakfast / Coffee</t>
+          <t>@blendgreenness</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Lunch / Sandwiches</t>
         </is>
       </c>
       <c r="D64" s="21" t="inlineStr">
         <is>
-          <t>350m</t>
+          <t>450m</t>
         </is>
       </c>
       <c r="E64" s="21" t="inlineStr">
         <is>
+          <t>6 min</t>
+        </is>
+      </c>
+      <c r="F64" s="21" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="G64" s="21" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" hidden="1">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Bistro Margaux</t>
+        </is>
+      </c>
+      <c r="B65" s="17" t="inlineStr">
+        <is>
+          <t>@bistro_margaux</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Dinner / French Bistro</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>2km</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
           <t>4 min</t>
         </is>
       </c>
-      <c r="F64" s="21" t="inlineStr">
-        <is>
-          <t>Walk</t>
-        </is>
-      </c>
-      <c r="G64" s="21" t="inlineStr">
-        <is>
-          <t>Breakfast &amp; Cafés</t>
-        </is>
-      </c>
-      <c r="H64" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" hidden="1">
-      <c r="A65" s="22" t="inlineStr">
-        <is>
-          <t>Blend Greenness</t>
-        </is>
-      </c>
-      <c r="B65" s="14" t="inlineStr">
-        <is>
-          <t>@blendgreenness</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>Lunch / Sandwiches</t>
-        </is>
-      </c>
-      <c r="D65" s="21" t="inlineStr">
-        <is>
-          <t>450m</t>
-        </is>
-      </c>
-      <c r="E65" s="21" t="inlineStr">
-        <is>
-          <t>6 min</t>
-        </is>
-      </c>
-      <c r="F65" s="21" t="inlineStr">
-        <is>
-          <t>Walk</t>
-        </is>
-      </c>
-      <c r="G65" s="21" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="H65" t="inlineStr">
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Dinner</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>Bistro Margaux</t>
-        </is>
-      </c>
-      <c r="B66" s="17" t="inlineStr">
-        <is>
-          <t>@bistro_margaux</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>Dinner / French Bistro</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>2km</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="inlineStr">
-        <is>
-          <t>4 min</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>Dinner</t>
+      <c r="A66" s="22" t="inlineStr">
+        <is>
+          <t>Frankies Gelato</t>
+        </is>
+      </c>
+      <c r="B66" s="23" t="inlineStr">
+        <is>
+          <t>@frankiesgelato</t>
+        </is>
+      </c>
+      <c r="C66" s="21" t="inlineStr">
+        <is>
+          <t>Gelato</t>
+        </is>
+      </c>
+      <c r="D66" s="21" t="inlineStr">
+        <is>
+          <t>2.1km</t>
+        </is>
+      </c>
+      <c r="E66" s="21" t="inlineStr">
+        <is>
+          <t>7 min</t>
+        </is>
+      </c>
+      <c r="F66" s="21" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="G66" s="21" t="inlineStr">
+        <is>
+          <t>Dessert</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -3191,40 +3207,192 @@
     <row r="67">
       <c r="A67" s="22" t="inlineStr">
         <is>
-          <t>Frankies Gelato</t>
-        </is>
-      </c>
-      <c r="B67" s="23" t="inlineStr">
-        <is>
-          <t>@frankiesgelato</t>
-        </is>
-      </c>
+          <t>Sushi Daruma</t>
+        </is>
+      </c>
+      <c r="B67" s="21" t="n"/>
       <c r="C67" s="21" t="inlineStr">
         <is>
-          <t>Gelato</t>
+          <t>Japanese Sushi</t>
         </is>
       </c>
       <c r="D67" s="21" t="inlineStr">
         <is>
+          <t>450m</t>
+        </is>
+      </c>
+      <c r="E67" s="21" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="F67" s="21" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="G67" s="21" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="22" t="inlineStr">
+        <is>
+          <t>Miami Rice</t>
+        </is>
+      </c>
+      <c r="B68" s="21" t="n"/>
+      <c r="C68" s="21" t="inlineStr">
+        <is>
+          <t>Malaysian Chinese</t>
+        </is>
+      </c>
+      <c r="D68" s="21" t="inlineStr">
+        <is>
+          <t>600m</t>
+        </is>
+      </c>
+      <c r="E68" s="21" t="inlineStr">
+        <is>
+          <t>9 min</t>
+        </is>
+      </c>
+      <c r="F68" s="21" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="G68" s="21" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="22" t="inlineStr">
+        <is>
+          <t>Terronia Cocktail Bar</t>
+        </is>
+      </c>
+      <c r="B69" s="21" t="inlineStr">
+        <is>
+          <t>@terronia.burleigh</t>
+        </is>
+      </c>
+      <c r="C69" s="21" t="inlineStr">
+        <is>
+          <t>Cocktail Bar</t>
+        </is>
+      </c>
+      <c r="D69" s="21" t="inlineStr">
+        <is>
           <t>2.1km</t>
         </is>
       </c>
-      <c r="E67" s="21" t="inlineStr">
-        <is>
-          <t>7 min</t>
-        </is>
-      </c>
-      <c r="F67" s="21" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
-      <c r="G67" s="21" t="inlineStr">
-        <is>
-          <t>Dessert</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
+      <c r="E69" s="21" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="F69" s="21" t="inlineStr">
+        <is>
+          <t>Drive</t>
+        </is>
+      </c>
+      <c r="G69" s="21" t="inlineStr">
+        <is>
+          <t>Drinks</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="22" t="inlineStr">
+        <is>
+          <t>Dalas Kitchen - Salad Bar</t>
+        </is>
+      </c>
+      <c r="B70" s="21" t="inlineStr">
+        <is>
+          <t>@dalas_kitchen</t>
+        </is>
+      </c>
+      <c r="C70" s="21" t="inlineStr">
+        <is>
+          <t>Breakfast</t>
+        </is>
+      </c>
+      <c r="D70" s="21" t="inlineStr">
+        <is>
+          <t>450m</t>
+        </is>
+      </c>
+      <c r="E70" s="21" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="F70" s="21" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="G70" s="21" t="inlineStr">
+        <is>
+          <t>Breakfast &amp; Cafés</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="22" t="inlineStr">
+        <is>
+          <t>Krunch Cluck</t>
+        </is>
+      </c>
+      <c r="B71" s="21" t="inlineStr">
+        <is>
+          <t>@krunchcluck</t>
+        </is>
+      </c>
+      <c r="C71" s="21" t="inlineStr">
+        <is>
+          <t>Korean Chicken</t>
+        </is>
+      </c>
+      <c r="D71" s="21" t="inlineStr">
+        <is>
+          <t>450m</t>
+        </is>
+      </c>
+      <c r="E71" s="21" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="F71" s="21" t="inlineStr">
+        <is>
+          <t>Walk</t>
+        </is>
+      </c>
+      <c r="G71" s="21" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>

</xml_diff>